<commit_message>
fix(dosing): correct pediatric renal dosing rules and add adult calculation module with CG calculator
</commit_message>
<xml_diff>
--- a/药品规则数据模板_思福妥_思福诺.xlsx
+++ b/药品规则数据模板_思福妥_思福诺.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T21"/>
+  <dimension ref="A1:T26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -513,10 +513,10 @@
         <v>说明书</v>
       </c>
       <c r="Q2" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R2" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表3</v>
       </c>
       <c r="S2" t="str">
         <v>医学事务部</v>
@@ -575,10 +575,10 @@
         <v>说明书</v>
       </c>
       <c r="Q3" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R3" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表3</v>
       </c>
       <c r="S3" t="str">
         <v>医学事务部</v>
@@ -628,7 +628,7 @@
         <v>1</v>
       </c>
       <c r="N4" t="str">
-        <v>PMA &gt;44-52周且eCrCL &gt; 50</v>
+        <v>PMA 45 ~ &lt;53周且eCrCL &gt; 50</v>
       </c>
       <c r="O4" t="str">
         <v>有肾损伤体征的&lt;3月龄患儿无推荐剂量，禁止计算</v>
@@ -637,10 +637,10 @@
         <v>说明书</v>
       </c>
       <c r="Q4" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R4" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表3</v>
       </c>
       <c r="S4" t="str">
         <v>医学事务部</v>
@@ -699,10 +699,10 @@
         <v>说明书</v>
       </c>
       <c r="Q5" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R5" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表6</v>
       </c>
       <c r="S5" t="str">
         <v>医学事务部</v>
@@ -761,10 +761,10 @@
         <v>说明书</v>
       </c>
       <c r="Q6" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R6" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表6</v>
       </c>
       <c r="S6" t="str">
         <v>医学事务部</v>
@@ -823,10 +823,10 @@
         <v>说明书</v>
       </c>
       <c r="Q7" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R7" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表2</v>
       </c>
       <c r="S7" t="str">
         <v>医学事务部</v>
@@ -855,10 +855,10 @@
         <v>mg/kg</v>
       </c>
       <c r="G8">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H8">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I8" t="str">
         <v>q8h</v>
@@ -885,10 +885,10 @@
         <v>说明书</v>
       </c>
       <c r="Q8" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R8" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表5</v>
       </c>
       <c r="S8" t="str">
         <v>医学事务部</v>
@@ -917,10 +917,10 @@
         <v>mg/kg</v>
       </c>
       <c r="G9">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H9">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I9" t="str">
         <v>q12h</v>
@@ -947,10 +947,10 @@
         <v>说明书</v>
       </c>
       <c r="Q9" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R9" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表5</v>
       </c>
       <c r="S9" t="str">
         <v>医学事务部</v>
@@ -1009,10 +1009,10 @@
         <v>说明书</v>
       </c>
       <c r="Q10" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R10" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表2</v>
       </c>
       <c r="S10" t="str">
         <v>医学事务部</v>
@@ -1041,10 +1041,10 @@
         <v>mg/kg</v>
       </c>
       <c r="G11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I11" t="str">
         <v>q8h</v>
@@ -1071,10 +1071,10 @@
         <v>说明书</v>
       </c>
       <c r="Q11" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R11" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表5</v>
       </c>
       <c r="S11" t="str">
         <v>医学事务部</v>
@@ -1103,10 +1103,10 @@
         <v>mg/kg</v>
       </c>
       <c r="G12">
-        <v>15</v>
+        <v>18.75</v>
       </c>
       <c r="H12">
-        <v>15</v>
+        <v>18.75</v>
       </c>
       <c r="I12" t="str">
         <v>q12h</v>
@@ -1133,10 +1133,10 @@
         <v>说明书</v>
       </c>
       <c r="Q12" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R12" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表5</v>
       </c>
       <c r="S12" t="str">
         <v>医学事务部</v>
@@ -1195,10 +1195,10 @@
         <v>说明书</v>
       </c>
       <c r="Q13" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R13" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表2</v>
       </c>
       <c r="S13" t="str">
         <v>医学事务部</v>
@@ -1227,10 +1227,10 @@
         <v>mg/kg</v>
       </c>
       <c r="G14">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H14">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I14" t="str">
         <v>q8h</v>
@@ -1257,10 +1257,10 @@
         <v>说明书</v>
       </c>
       <c r="Q14" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R14" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表5</v>
       </c>
       <c r="S14" t="str">
         <v>医学事务部</v>
@@ -1289,10 +1289,10 @@
         <v>mg/kg</v>
       </c>
       <c r="G15">
-        <v>15</v>
+        <v>18.75</v>
       </c>
       <c r="H15">
-        <v>15</v>
+        <v>18.75</v>
       </c>
       <c r="I15" t="str">
         <v>q12h</v>
@@ -1319,10 +1319,10 @@
         <v>说明书</v>
       </c>
       <c r="Q15" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R15" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表5</v>
       </c>
       <c r="S15" t="str">
         <v>医学事务部</v>
@@ -1351,10 +1351,10 @@
         <v>mg/kg</v>
       </c>
       <c r="G16">
-        <v>15</v>
+        <v>18.75</v>
       </c>
       <c r="H16">
-        <v>15</v>
+        <v>18.75</v>
       </c>
       <c r="I16" t="str">
         <v>q24h</v>
@@ -1381,10 +1381,10 @@
         <v>说明书</v>
       </c>
       <c r="Q16" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R16" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表5</v>
       </c>
       <c r="S16" t="str">
         <v>医学事务部</v>
@@ -1413,16 +1413,16 @@
         <v>mg/kg</v>
       </c>
       <c r="G17">
-        <v>15</v>
+        <v>18.75</v>
       </c>
       <c r="H17">
-        <v>15</v>
+        <v>18.75</v>
       </c>
       <c r="I17" t="str">
         <v>q48h</v>
       </c>
       <c r="J17">
-        <v>375</v>
+        <v>750</v>
       </c>
       <c r="K17" t="b">
         <v>1</v>
@@ -1443,10 +1443,10 @@
         <v>说明书</v>
       </c>
       <c r="Q17" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R17" t="str">
-        <v>说明书/剂量卡</v>
+        <v>说明书表5</v>
       </c>
       <c r="S17" t="str">
         <v>医学事务部</v>
@@ -1505,7 +1505,7 @@
         <v>说明书</v>
       </c>
       <c r="Q18" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R18" t="str">
         <v>说明书/剂量卡</v>
@@ -1567,7 +1567,7 @@
         <v>说明书</v>
       </c>
       <c r="Q19" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R19" t="str">
         <v>说明书/剂量卡</v>
@@ -1629,7 +1629,7 @@
         <v>说明书</v>
       </c>
       <c r="Q20" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R20" t="str">
         <v>说明书/剂量卡</v>
@@ -1691,7 +1691,7 @@
         <v>说明书</v>
       </c>
       <c r="Q21" t="str">
-        <v>20210602</v>
+        <v>20250416</v>
       </c>
       <c r="R21" t="str">
         <v>说明书/剂量卡</v>
@@ -1703,9 +1703,319 @@
         <v>2026-07-07</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>CAZ_AVI</v>
+      </c>
+      <c r="B22" t="str">
+        <v>思福妥</v>
+      </c>
+      <c r="C22" t="str">
+        <v>头孢他啶阿维巴坦</v>
+      </c>
+      <c r="D22" t="str">
+        <v>成人</v>
+      </c>
+      <c r="E22" t="str">
+        <v>不限</v>
+      </c>
+      <c r="F22" t="str">
+        <v>mg</v>
+      </c>
+      <c r="G22">
+        <v>2000</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22" t="str">
+        <v>q8h</v>
+      </c>
+      <c r="J22">
+        <v>6000</v>
+      </c>
+      <c r="K22" t="b">
+        <v>1</v>
+      </c>
+      <c r="L22" t="str">
+        <v>重症监测清除率</v>
+      </c>
+      <c r="M22" t="b">
+        <v>1</v>
+      </c>
+      <c r="N22" t="str">
+        <v>成人且eCrCL &gt; 50</v>
+      </c>
+      <c r="O22" t="str">
+        <v>无特别警告</v>
+      </c>
+      <c r="P22" t="str">
+        <v>说明书</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>20250416</v>
+      </c>
+      <c r="R22" t="str">
+        <v>说明书表2/表5</v>
+      </c>
+      <c r="S22" t="str">
+        <v>医学事务部</v>
+      </c>
+      <c r="T22" t="str">
+        <v>2026-07-10</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>CAZ_AVI</v>
+      </c>
+      <c r="B23" t="str">
+        <v>思福妥</v>
+      </c>
+      <c r="C23" t="str">
+        <v>头孢他啶阿维巴坦</v>
+      </c>
+      <c r="D23" t="str">
+        <v>成人</v>
+      </c>
+      <c r="E23" t="str">
+        <v>不限</v>
+      </c>
+      <c r="F23" t="str">
+        <v>mg</v>
+      </c>
+      <c r="G23">
+        <v>1000</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23" t="str">
+        <v>q8h</v>
+      </c>
+      <c r="J23">
+        <v>3000</v>
+      </c>
+      <c r="K23" t="b">
+        <v>1</v>
+      </c>
+      <c r="L23" t="str">
+        <v>重症监测清除率</v>
+      </c>
+      <c r="M23" t="b">
+        <v>1</v>
+      </c>
+      <c r="N23" t="str">
+        <v>成人且eCrCL 31-50</v>
+      </c>
+      <c r="O23" t="str">
+        <v>无特别警告</v>
+      </c>
+      <c r="P23" t="str">
+        <v>说明书</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>20250416</v>
+      </c>
+      <c r="R23" t="str">
+        <v>说明书表2/表5</v>
+      </c>
+      <c r="S23" t="str">
+        <v>医学事务部</v>
+      </c>
+      <c r="T23" t="str">
+        <v>2026-07-10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>CAZ_AVI</v>
+      </c>
+      <c r="B24" t="str">
+        <v>思福妥</v>
+      </c>
+      <c r="C24" t="str">
+        <v>头孢他啶阿维巴坦</v>
+      </c>
+      <c r="D24" t="str">
+        <v>成人</v>
+      </c>
+      <c r="E24" t="str">
+        <v>不限</v>
+      </c>
+      <c r="F24" t="str">
+        <v>mg</v>
+      </c>
+      <c r="G24">
+        <v>750</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24" t="str">
+        <v>q12h</v>
+      </c>
+      <c r="J24">
+        <v>1500</v>
+      </c>
+      <c r="K24" t="b">
+        <v>1</v>
+      </c>
+      <c r="L24" t="str">
+        <v>重症监测清除率</v>
+      </c>
+      <c r="M24" t="b">
+        <v>1</v>
+      </c>
+      <c r="N24" t="str">
+        <v>成人且eCrCL 16-30</v>
+      </c>
+      <c r="O24" t="str">
+        <v>无特别警告</v>
+      </c>
+      <c r="P24" t="str">
+        <v>说明书</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>20250416</v>
+      </c>
+      <c r="R24" t="str">
+        <v>说明书表2/表5</v>
+      </c>
+      <c r="S24" t="str">
+        <v>医学事务部</v>
+      </c>
+      <c r="T24" t="str">
+        <v>2026-07-10</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>CAZ_AVI</v>
+      </c>
+      <c r="B25" t="str">
+        <v>思福妥</v>
+      </c>
+      <c r="C25" t="str">
+        <v>头孢他啶阿维巴坦</v>
+      </c>
+      <c r="D25" t="str">
+        <v>成人</v>
+      </c>
+      <c r="E25" t="str">
+        <v>不限</v>
+      </c>
+      <c r="F25" t="str">
+        <v>mg</v>
+      </c>
+      <c r="G25">
+        <v>750</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25" t="str">
+        <v>q24h</v>
+      </c>
+      <c r="J25">
+        <v>750</v>
+      </c>
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+      <c r="L25" t="str">
+        <v>重症监测清除率</v>
+      </c>
+      <c r="M25" t="b">
+        <v>1</v>
+      </c>
+      <c r="N25" t="str">
+        <v>成人且eCrCL 6-15</v>
+      </c>
+      <c r="O25" t="str">
+        <v>无特别警告</v>
+      </c>
+      <c r="P25" t="str">
+        <v>说明书</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>20250416</v>
+      </c>
+      <c r="R25" t="str">
+        <v>说明书表2/表5</v>
+      </c>
+      <c r="S25" t="str">
+        <v>医学事务部</v>
+      </c>
+      <c r="T25" t="str">
+        <v>2026-07-10</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>CAZ_AVI</v>
+      </c>
+      <c r="B26" t="str">
+        <v>思福妥</v>
+      </c>
+      <c r="C26" t="str">
+        <v>头孢他啶阿维巴坦</v>
+      </c>
+      <c r="D26" t="str">
+        <v>成人</v>
+      </c>
+      <c r="E26" t="str">
+        <v>不限</v>
+      </c>
+      <c r="F26" t="str">
+        <v>mg</v>
+      </c>
+      <c r="G26">
+        <v>750</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26" t="str">
+        <v>q48h</v>
+      </c>
+      <c r="J26">
+        <v>750</v>
+      </c>
+      <c r="K26" t="b">
+        <v>1</v>
+      </c>
+      <c r="L26" t="str">
+        <v>重症监测清除率</v>
+      </c>
+      <c r="M26" t="b">
+        <v>1</v>
+      </c>
+      <c r="N26" t="str">
+        <v>成人且ESRD</v>
+      </c>
+      <c r="O26" t="str">
+        <v>在血液透析当日，应在血液透析完成后给予本品</v>
+      </c>
+      <c r="P26" t="str">
+        <v>说明书</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>20250416</v>
+      </c>
+      <c r="R26" t="str">
+        <v>说明书表2/表5</v>
+      </c>
+      <c r="S26" t="str">
+        <v>医学事务部</v>
+      </c>
+      <c r="T26" t="str">
+        <v>2026-07-10</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T26"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1771,7 +2081,7 @@
         <v>剂量调整</v>
       </c>
       <c r="D3">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="E3" t="str">
         <v>q8h</v>
@@ -1794,7 +2104,7 @@
         <v>剂量调整且给药间隔延长</v>
       </c>
       <c r="D4">
-        <v>0.3</v>
+        <v>0.375</v>
       </c>
       <c r="E4" t="str">
         <v>q12h</v>
@@ -1817,7 +2127,7 @@
         <v>剂量调整且给药间隔延长</v>
       </c>
       <c r="D5">
-        <v>0.3</v>
+        <v>0.375</v>
       </c>
       <c r="E5" t="str">
         <v>q24h</v>
@@ -1840,7 +2150,7 @@
         <v>剂量调整且给药间隔延长</v>
       </c>
       <c r="D6">
-        <v>0.3</v>
+        <v>0.375</v>
       </c>
       <c r="E6" t="str">
         <v>q48h</v>

</xml_diff>